<commit_message>
chore: actualización semanal 2026-09-07
</commit_message>
<xml_diff>
--- a/seguimiento_legislativo.xlsx
+++ b/seguimiento_legislativo.xlsx
@@ -575,47 +575,47 @@
     <row r="2" ht="70" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>16553-12</t>
+          <t>18216-05</t>
         </is>
       </c>
       <c r="B2" s="11" t="inlineStr">
         <is>
-          <t>Fortalece y mejora la eficacia de la fiscalización y el cumplimiento de la regulación ambiental a cargo de la Superintendencia del Medio Ambiente, y regula otras materias que indica</t>
+          <t>Para la reconstrucción nacional y el desarrollo económico y social</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>18/08/2026</t>
+          <t>01/09/2026</t>
         </is>
       </c>
       <c r="D2" s="11" t="inlineStr">
         <is>
-          <t>Segundo trámite constitucional / Senado — Cuenta del Mensaje 267-374 que retira y hace presente la urgencia Simple</t>
+          <t>Trámite en Tribunal Constitucional / C.Diputados — Oficio N°2059/2026. Respuesta Ministerio de Hacienda</t>
         </is>
       </c>
       <c r="E2" s="4" t="inlineStr">
         <is>
-          <t>Simple</t>
+          <t>Discusión inmediata</t>
         </is>
       </c>
       <c r="F2" s="4" t="inlineStr">
         <is>
-          <t>Senado</t>
+          <t>Cámara</t>
         </is>
       </c>
       <c r="G2" s="11" t="inlineStr">
         <is>
-          <t>Medio Ambiente, Cambio Climático y Bienes Nacionales</t>
+          <t>Ingreso fallo del Tribunal Constitucional</t>
         </is>
       </c>
       <c r="H2" s="4" t="inlineStr">
         <is>
-          <t>Miércoles 10 de Enero, 2024</t>
+          <t>Miércoles 22 de Abril, 2026</t>
         </is>
       </c>
       <c r="I2" s="11" t="inlineStr">
         <is>
-          <t>Segundo trámite constitucional / Senado</t>
+          <t>Trámite en Tribunal Constitucional / C.Diputados — Oficio</t>
         </is>
       </c>
       <c r="J2" s="4" t="inlineStr">
@@ -630,54 +630,54 @@
       </c>
       <c r="L2" s="11" t="inlineStr">
         <is>
-          <t>Ministerio del Medio Ambiente</t>
+          <t>Ministerio de Hacienda</t>
         </is>
       </c>
     </row>
     <row r="3" ht="70" customHeight="1">
       <c r="A3" s="5" t="inlineStr">
         <is>
-          <t>18216-05</t>
+          <t>16553-12</t>
         </is>
       </c>
       <c r="B3" s="12" t="inlineStr">
         <is>
-          <t>Para la reconstrucción nacional y el desarrollo económico y social</t>
+          <t>Fortalece y mejora la eficacia de la fiscalización y el cumplimiento de la regulación ambiental a cargo de la Superintendencia del Medio Ambiente, y regula otras materias que indica</t>
         </is>
       </c>
       <c r="C3" s="7" t="inlineStr">
         <is>
-          <t>17/08/2026</t>
+          <t>18/08/2026</t>
         </is>
       </c>
       <c r="D3" s="12" t="inlineStr">
         <is>
-          <t>Trámite finalización en Cámara de Origen / C.Diputados — Cuenta, Copia autorizada de una resolución del Tribunal Constitucional mediante la cual prorroga por diez días el plazo para resolver el requerimiento de inconstitucionalidad presentado respecto del proyecto.</t>
+          <t>Segundo trámite constitucional / Senado — Cuenta del Mensaje 267-374 que retira y hace presente la urgencia Simple</t>
         </is>
       </c>
       <c r="E3" s="7" t="inlineStr">
         <is>
-          <t>Discusión inmediata</t>
+          <t>Simple</t>
         </is>
       </c>
       <c r="F3" s="7" t="inlineStr">
         <is>
-          <t>Cámara</t>
+          <t>Senado</t>
         </is>
       </c>
       <c r="G3" s="12" t="inlineStr">
         <is>
-          <t>Ingreso fallo del Tribunal Constitucional</t>
+          <t>Medio Ambiente, Cambio Climático y Bienes Nacionales</t>
         </is>
       </c>
       <c r="H3" s="7" t="inlineStr">
         <is>
-          <t>Miércoles 22 de Abril, 2026</t>
+          <t>Miércoles 10 de Enero, 2024</t>
         </is>
       </c>
       <c r="I3" s="12" t="inlineStr">
         <is>
-          <t>Trámite finalización en Cámara de Origen / C.Diputados</t>
+          <t>Segundo trámite constitucional / Senado</t>
         </is>
       </c>
       <c r="J3" s="7" t="inlineStr">
@@ -692,7 +692,7 @@
       </c>
       <c r="L3" s="12" t="inlineStr">
         <is>
-          <t>Ministerio de Hacienda</t>
+          <t>Ministerio del Medio Ambiente</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: actualización semanal 2026-09-14
</commit_message>
<xml_diff>
--- a/seguimiento_legislativo.xlsx
+++ b/seguimiento_legislativo.xlsx
@@ -575,47 +575,47 @@
     <row r="2" ht="70" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>18216-05</t>
+          <t>16553-12</t>
         </is>
       </c>
       <c r="B2" s="11" t="inlineStr">
         <is>
-          <t>Para la reconstrucción nacional y el desarrollo económico y social</t>
+          <t>Fortalece y mejora la eficacia de la fiscalización y el cumplimiento de la regulación ambiental a cargo de la Superintendencia del Medio Ambiente, y regula otras materias que indica</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>01/09/2026</t>
+          <t>08/09/2026</t>
         </is>
       </c>
       <c r="D2" s="11" t="inlineStr">
         <is>
-          <t>Trámite en Tribunal Constitucional / C.Diputados — Oficio N°2059/2026. Respuesta Ministerio de Hacienda</t>
+          <t>Segundo trámite constitucional / Senado — Cuenta del Mensaje 311-374 que retira y hace presente la urgencia Simple</t>
         </is>
       </c>
       <c r="E2" s="4" t="inlineStr">
         <is>
-          <t>Discusión inmediata</t>
+          <t>Simple</t>
         </is>
       </c>
       <c r="F2" s="4" t="inlineStr">
         <is>
-          <t>Cámara</t>
+          <t>Senado</t>
         </is>
       </c>
       <c r="G2" s="11" t="inlineStr">
         <is>
-          <t>Ingreso fallo del Tribunal Constitucional</t>
+          <t>Medio Ambiente, Cambio Climático y Bienes Nacionales</t>
         </is>
       </c>
       <c r="H2" s="4" t="inlineStr">
         <is>
-          <t>Miércoles 22 de Abril, 2026</t>
+          <t>Miércoles 10 de Enero, 2024</t>
         </is>
       </c>
       <c r="I2" s="11" t="inlineStr">
         <is>
-          <t>Trámite en Tribunal Constitucional / C.Diputados — Oficio</t>
+          <t>Segundo trámite constitucional / Senado</t>
         </is>
       </c>
       <c r="J2" s="4" t="inlineStr">
@@ -630,29 +630,29 @@
       </c>
       <c r="L2" s="11" t="inlineStr">
         <is>
-          <t>Ministerio de Hacienda</t>
+          <t>Ministerio del Medio Ambiente</t>
         </is>
       </c>
     </row>
     <row r="3" ht="70" customHeight="1">
       <c r="A3" s="5" t="inlineStr">
         <is>
-          <t>16553-12</t>
+          <t>16.552-12</t>
         </is>
       </c>
       <c r="B3" s="12" t="inlineStr">
         <is>
-          <t>Fortalece y mejora la eficacia de la fiscalización y el cumplimiento de la regulación ambiental a cargo de la Superintendencia del Medio Ambiente, y regula otras materias que indica</t>
+          <t>Modifica diversos cuerpos legales, con el objeto de fortalecer la institucionalidad ambiental y mejorar su eficiencia</t>
         </is>
       </c>
       <c r="C3" s="7" t="inlineStr">
         <is>
-          <t>18/08/2026</t>
+          <t>07/09/2026</t>
         </is>
       </c>
       <c r="D3" s="12" t="inlineStr">
         <is>
-          <t>Segundo trámite constitucional / Senado — Cuenta del Mensaje 267-374 que retira y hace presente la urgencia Simple</t>
+          <t>Segundo trámite constitucional / C.Diputados — Cuenta del Mensaje 302-374 que retira y hace presente la urgencia Simple</t>
         </is>
       </c>
       <c r="E3" s="7" t="inlineStr">
@@ -662,64 +662,64 @@
       </c>
       <c r="F3" s="7" t="inlineStr">
         <is>
+          <t>Cámara</t>
+        </is>
+      </c>
+      <c r="G3" s="12" t="inlineStr">
+        <is>
+          <t>Primer informe de comisión Medio Ambiente y Recursos Naturales</t>
+        </is>
+      </c>
+      <c r="H3" s="7" t="inlineStr">
+        <is>
+          <t>10 de enero de 2024</t>
+        </is>
+      </c>
+      <c r="I3" s="12" t="inlineStr">
+        <is>
+          <t>Segundo trámite constitucional / C.Diputados</t>
+        </is>
+      </c>
+      <c r="J3" s="7" t="inlineStr">
+        <is>
+          <t>Mensaje</t>
+        </is>
+      </c>
+      <c r="K3" s="7" t="inlineStr">
+        <is>
           <t>Senado</t>
         </is>
       </c>
-      <c r="G3" s="12" t="inlineStr">
-        <is>
-          <t>Medio Ambiente, Cambio Climático y Bienes Nacionales</t>
-        </is>
-      </c>
-      <c r="H3" s="7" t="inlineStr">
-        <is>
-          <t>Miércoles 10 de Enero, 2024</t>
-        </is>
-      </c>
-      <c r="I3" s="12" t="inlineStr">
-        <is>
-          <t>Segundo trámite constitucional / Senado</t>
-        </is>
-      </c>
-      <c r="J3" s="7" t="inlineStr">
-        <is>
-          <t>Mensaje</t>
-        </is>
-      </c>
-      <c r="K3" s="7" t="inlineStr">
-        <is>
-          <t>C.Diputados</t>
-        </is>
-      </c>
       <c r="L3" s="12" t="inlineStr">
         <is>
-          <t>Ministerio del Medio Ambiente</t>
+          <t>Ministerio de Agricultura; Ministerio de Economía, Fomento y Turismo; Ministerio de Energía; Ministerio de Hacienda; Ministerio de Obras Públicas; Ministerio del Medio Ambiente</t>
         </is>
       </c>
     </row>
     <row r="4" ht="70" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>16.552-12</t>
+          <t>18216-05</t>
         </is>
       </c>
       <c r="B4" s="11" t="inlineStr">
         <is>
-          <t>Modifica diversos cuerpos legales, con el objeto de fortalecer la institucionalidad ambiental y mejorar su eficiencia</t>
+          <t>Para la reconstrucción nacional y el desarrollo económico y social</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>17/08/2026</t>
+          <t>01/09/2026</t>
         </is>
       </c>
       <c r="D4" s="11" t="inlineStr">
         <is>
-          <t>Segundo trámite constitucional / C.Diputados — Cuenta del Mensaje 262-374 que retira y hace presente la urgencia Simple</t>
+          <t>Trámite en Tribunal Constitucional / C.Diputados — Oficio N°2059/2026. Respuesta Ministerio de Hacienda</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>Simple</t>
+          <t>Discusión inmediata</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
@@ -729,17 +729,17 @@
       </c>
       <c r="G4" s="11" t="inlineStr">
         <is>
-          <t>Primer informe de comisión Medio Ambiente y Recursos Naturales</t>
+          <t>Ingreso fallo del Tribunal Constitucional</t>
         </is>
       </c>
       <c r="H4" s="4" t="inlineStr">
         <is>
-          <t>10 de enero de 2024</t>
+          <t>Miércoles 22 de Abril, 2026</t>
         </is>
       </c>
       <c r="I4" s="11" t="inlineStr">
         <is>
-          <t>Segundo trámite constitucional / C.Diputados</t>
+          <t>Trámite en Tribunal Constitucional / C.Diputados — Oficio</t>
         </is>
       </c>
       <c r="J4" s="4" t="inlineStr">
@@ -749,12 +749,12 @@
       </c>
       <c r="K4" s="4" t="inlineStr">
         <is>
-          <t>Senado</t>
+          <t>C.Diputados</t>
         </is>
       </c>
       <c r="L4" s="11" t="inlineStr">
         <is>
-          <t>Ministerio de Agricultura; Ministerio de Economía, Fomento y Turismo; Ministerio de Energía; Ministerio de Hacienda; Ministerio de Obras Públicas; Ministerio del Medio Ambiente</t>
+          <t>Ministerio de Hacienda</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: actualización semanal 2026-09-21
</commit_message>
<xml_diff>
--- a/seguimiento_legislativo.xlsx
+++ b/seguimiento_legislativo.xlsx
@@ -575,22 +575,22 @@
     <row r="2" ht="70" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>16553-12</t>
+          <t>16.552-12</t>
         </is>
       </c>
       <c r="B2" s="11" t="inlineStr">
         <is>
-          <t>Fortalece y mejora la eficacia de la fiscalización y el cumplimiento de la regulación ambiental a cargo de la Superintendencia del Medio Ambiente, y regula otras materias que indica</t>
+          <t>Modifica diversos cuerpos legales, con el objeto de fortalecer la institucionalidad ambiental y mejorar su eficiencia</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>08/09/2026</t>
+          <t>09/09/2026</t>
         </is>
       </c>
       <c r="D2" s="11" t="inlineStr">
         <is>
-          <t>Segundo trámite constitucional / Senado — Cuenta del Mensaje 311-374 que retira y hace presente la urgencia Simple</t>
+          <t>Segundo trámite constitucional / C.Diputados — S.E. el Presidente de la República retira la urgencia "simple", hecha presente para el despacho de proyecto. (320-374).</t>
         </is>
       </c>
       <c r="E2" s="4" t="inlineStr">
@@ -600,59 +600,59 @@
       </c>
       <c r="F2" s="4" t="inlineStr">
         <is>
+          <t>Cámara</t>
+        </is>
+      </c>
+      <c r="G2" s="11" t="inlineStr">
+        <is>
+          <t>Primer informe de comisión Medio Ambiente y Recursos Naturales</t>
+        </is>
+      </c>
+      <c r="H2" s="4" t="inlineStr">
+        <is>
+          <t>10 de enero de 2024</t>
+        </is>
+      </c>
+      <c r="I2" s="11" t="inlineStr">
+        <is>
+          <t>Segundo trámite constitucional / C.Diputados — Oficio</t>
+        </is>
+      </c>
+      <c r="J2" s="4" t="inlineStr">
+        <is>
+          <t>Mensaje</t>
+        </is>
+      </c>
+      <c r="K2" s="4" t="inlineStr">
+        <is>
           <t>Senado</t>
         </is>
       </c>
-      <c r="G2" s="11" t="inlineStr">
-        <is>
-          <t>Medio Ambiente, Cambio Climático y Bienes Nacionales</t>
-        </is>
-      </c>
-      <c r="H2" s="4" t="inlineStr">
-        <is>
-          <t>Miércoles 10 de Enero, 2024</t>
-        </is>
-      </c>
-      <c r="I2" s="11" t="inlineStr">
-        <is>
-          <t>Segundo trámite constitucional / Senado</t>
-        </is>
-      </c>
-      <c r="J2" s="4" t="inlineStr">
-        <is>
-          <t>Mensaje</t>
-        </is>
-      </c>
-      <c r="K2" s="4" t="inlineStr">
-        <is>
-          <t>C.Diputados</t>
-        </is>
-      </c>
       <c r="L2" s="11" t="inlineStr">
         <is>
-          <t>Ministerio del Medio Ambiente</t>
+          <t>Ministerio de Agricultura; Ministerio de Economía, Fomento y Turismo; Ministerio de Energía; Ministerio de Hacienda; Ministerio de Obras Públicas; Ministerio del Medio Ambiente</t>
         </is>
       </c>
     </row>
     <row r="3" ht="70" customHeight="1">
       <c r="A3" s="5" t="inlineStr">
         <is>
-          <t>16.552-12</t>
+          <t>16553-12</t>
         </is>
       </c>
       <c r="B3" s="12" t="inlineStr">
         <is>
-          <t>Modifica diversos cuerpos legales, con el objeto de fortalecer la institucionalidad ambiental y mejorar su eficiencia</t>
+          <t>Fortalece y mejora la eficacia de la fiscalización y el cumplimiento de la regulación ambiental a cargo de la Superintendencia del Medio Ambiente, y regula otras materias que indica</t>
         </is>
       </c>
       <c r="C3" s="7" t="inlineStr">
         <is>
-          <t>07/09/2026</t>
+          <t>08/09/2026</t>
         </is>
       </c>
       <c r="D3" s="12" t="inlineStr">
         <is>
-          <t>Segundo trámite constitucional / C.Diputados — Cuenta del Mensaje 302-374 que retira y hace presente la urgencia Simple</t>
+          <t>Segundo trámite constitucional / Senado — Cuenta del Mensaje 311-374 que retira y hace presente la urgencia Simple</t>
         </is>
       </c>
       <c r="E3" s="7" t="inlineStr">
@@ -662,22 +662,22 @@
       </c>
       <c r="F3" s="7" t="inlineStr">
         <is>
-          <t>Cámara</t>
+          <t>Senado</t>
         </is>
       </c>
       <c r="G3" s="12" t="inlineStr">
         <is>
-          <t>Primer informe de comisión Medio Ambiente y Recursos Naturales</t>
+          <t>Medio Ambiente, Cambio Climático y Bienes Nacionales</t>
         </is>
       </c>
       <c r="H3" s="7" t="inlineStr">
         <is>
-          <t>10 de enero de 2024</t>
+          <t>Miércoles 10 de Enero, 2024</t>
         </is>
       </c>
       <c r="I3" s="12" t="inlineStr">
         <is>
-          <t>Segundo trámite constitucional / C.Diputados</t>
+          <t>Segundo trámite constitucional / Senado</t>
         </is>
       </c>
       <c r="J3" s="7" t="inlineStr">
@@ -687,12 +687,12 @@
       </c>
       <c r="K3" s="7" t="inlineStr">
         <is>
-          <t>Senado</t>
+          <t>C.Diputados</t>
         </is>
       </c>
       <c r="L3" s="12" t="inlineStr">
         <is>
-          <t>Ministerio de Agricultura; Ministerio de Economía, Fomento y Turismo; Ministerio de Energía; Ministerio de Hacienda; Ministerio de Obras Públicas; Ministerio del Medio Ambiente</t>
+          <t>Ministerio del Medio Ambiente</t>
         </is>
       </c>
     </row>
@@ -709,12 +709,12 @@
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>01/09/2026</t>
+          <t>07/09/2026</t>
         </is>
       </c>
       <c r="D4" s="11" t="inlineStr">
         <is>
-          <t>Trámite en Tribunal Constitucional / C.Diputados — Oficio N°2059/2026. Respuesta Ministerio de Hacienda</t>
+          <t>Trámite en Tribunal Constitucional / C.Diputados — Cuenta, Oficio del Tribunal Constitucional por el cual remite copia autorizada de la sentencia definitiva recaída en el requerimiento de inconstitucionalidad presentado por S.E. el Presidente de la República, respecto del artículo 31 del proyecto. (343 -2026). BOLETÍN N° 18216-05. ROL N° 17892-26-CPT. RECHAZADO.</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">

</xml_diff>

<commit_message>
Agrega boletín 17196-17 (modificación Ley Sociedades Anónimas - DDHH empresas)
</commit_message>
<xml_diff>
--- a/seguimiento_legislativo.xlsx
+++ b/seguimiento_legislativo.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Seguimiento Legislativo" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Seguimiento Legislativo" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -496,7 +496,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L15"/>
+  <dimension ref="A1:L16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1437,6 +1437,68 @@
       <c r="L15" s="12" t="inlineStr">
         <is>
           <t>Isabel Allende Bussi</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>17196-17</t>
+        </is>
+      </c>
+      <c r="B16" s="11" t="inlineStr">
+        <is>
+          <t>Modifica la ley N° 18.046, Ley sobre Sociedades Anónimas, con el objeto de establecer obligaciones para promover la protección de derechos humanos, a las personas jurídicas que indica.</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>21/10/2024</t>
+        </is>
+      </c>
+      <c r="D16" s="11" t="inlineStr">
+        <is>
+          <t>Primer trámite constitucional / Senado — Cuenta de proyecto . Pasa a Comisión de Derechos Humanos, Nacionalidad y Ciudadanía</t>
+        </is>
+      </c>
+      <c r="E16" s="4" t="inlineStr">
+        <is>
+          <t>Sin urgencia</t>
+        </is>
+      </c>
+      <c r="F16" s="4" t="inlineStr">
+        <is>
+          <t>Senado</t>
+        </is>
+      </c>
+      <c r="G16" s="11" t="inlineStr">
+        <is>
+          <t>Derechos Humanos, Nacionalidad y Ciudadanía</t>
+        </is>
+      </c>
+      <c r="H16" s="4" t="inlineStr">
+        <is>
+          <t>Lunes 21 de Octubre, 2024</t>
+        </is>
+      </c>
+      <c r="I16" s="11" t="inlineStr">
+        <is>
+          <t>Primer trámite constitucional / Senado</t>
+        </is>
+      </c>
+      <c r="J16" s="4" t="inlineStr">
+        <is>
+          <t>Moción</t>
+        </is>
+      </c>
+      <c r="K16" s="4" t="inlineStr">
+        <is>
+          <t>Senado</t>
+        </is>
+      </c>
+      <c r="L16" s="11" t="inlineStr">
+        <is>
+          <t>Vodanovic Rojas, Paulina</t>
         </is>
       </c>
     </row>
@@ -1456,6 +1518,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A13" r:id="rId12"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A14" r:id="rId13"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A15" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A16" r:id="rId15"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: actualización semanal 2026-09-28
</commit_message>
<xml_diff>
--- a/seguimiento_legislativo.xlsx
+++ b/seguimiento_legislativo.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Seguimiento Legislativo" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Seguimiento Legislativo" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
chore: actualización semanal 2026-10-12
</commit_message>
<xml_diff>
--- a/seguimiento_legislativo.xlsx
+++ b/seguimiento_legislativo.xlsx
@@ -575,27 +575,27 @@
     <row r="2" ht="70" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>16.552-12</t>
+          <t>18216-05</t>
         </is>
       </c>
       <c r="B2" s="11" t="inlineStr">
         <is>
-          <t>Modifica diversos cuerpos legales, con el objeto de fortalecer la institucionalidad ambiental y mejorar su eficiencia</t>
+          <t>Para la reconstrucción nacional y el desarrollo económico y social</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>09/09/2026</t>
+          <t>09/10/2026</t>
         </is>
       </c>
       <c r="D2" s="11" t="inlineStr">
         <is>
-          <t>Segundo trámite constitucional / C.Diputados — S.E. el Presidente de la República retira la urgencia "simple", hecha presente para el despacho de proyecto. (320-374).</t>
+          <t>Trámite finalización en Cámara de Origen / C.Diputados — Oficio de ley al Ejecutivo .</t>
         </is>
       </c>
       <c r="E2" s="4" t="inlineStr">
         <is>
-          <t>Simple</t>
+          <t>Sin urgencia</t>
         </is>
       </c>
       <c r="F2" s="4" t="inlineStr">
@@ -605,17 +605,17 @@
       </c>
       <c r="G2" s="11" t="inlineStr">
         <is>
-          <t>Primer informe de comisión Medio Ambiente y Recursos Naturales</t>
+          <t>En espera de promulgación</t>
         </is>
       </c>
       <c r="H2" s="4" t="inlineStr">
         <is>
-          <t>10 de enero de 2024</t>
+          <t>Miércoles 22 de Abril, 2026</t>
         </is>
       </c>
       <c r="I2" s="11" t="inlineStr">
         <is>
-          <t>Segundo trámite constitucional / C.Diputados — Oficio</t>
+          <t>Trámite finalización en Cámara de Origen / C.Diputados — Oficio</t>
         </is>
       </c>
       <c r="J2" s="4" t="inlineStr">
@@ -625,12 +625,12 @@
       </c>
       <c r="K2" s="4" t="inlineStr">
         <is>
-          <t>Senado</t>
+          <t>C.Diputados</t>
         </is>
       </c>
       <c r="L2" s="11" t="inlineStr">
         <is>
-          <t>Ministerio de Agricultura; Ministerio de Economía, Fomento y Turismo; Ministerio de Energía; Ministerio de Hacienda; Ministerio de Obras Públicas; Ministerio del Medio Ambiente</t>
+          <t>Ministerio de Hacienda</t>
         </is>
       </c>
     </row>
@@ -647,12 +647,12 @@
       </c>
       <c r="C3" s="7" t="inlineStr">
         <is>
-          <t>08/09/2026</t>
+          <t>06/10/2026</t>
         </is>
       </c>
       <c r="D3" s="12" t="inlineStr">
         <is>
-          <t>Segundo trámite constitucional / Senado — Cuenta del Mensaje 311-374 que retira y hace presente la urgencia Simple</t>
+          <t>Segundo trámite constitucional / Senado — Cuenta del Mensaje 374-374 que retira y hace presente la urgencia Simple</t>
         </is>
       </c>
       <c r="E3" s="7" t="inlineStr">
@@ -699,27 +699,27 @@
     <row r="4" ht="70" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>18216-05</t>
+          <t>16.552-12</t>
         </is>
       </c>
       <c r="B4" s="11" t="inlineStr">
         <is>
-          <t>Para la reconstrucción nacional y el desarrollo económico y social</t>
+          <t>Modifica diversos cuerpos legales, con el objeto de fortalecer la institucionalidad ambiental y mejorar su eficiencia</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>07/09/2026</t>
+          <t>09/09/2026</t>
         </is>
       </c>
       <c r="D4" s="11" t="inlineStr">
         <is>
-          <t>Trámite en Tribunal Constitucional / C.Diputados — Cuenta, Oficio del Tribunal Constitucional por el cual remite copia autorizada de la sentencia definitiva recaída en el requerimiento de inconstitucionalidad presentado por S.E. el Presidente de la República, respecto del artículo 31 del proyecto. (343 -2026). BOLETÍN N° 18216-05. ROL N° 17892-26-CPT. RECHAZADO.</t>
+          <t>Segundo trámite constitucional / C.Diputados — S.E. el Presidente de la República retira la urgencia "simple", hecha presente para el despacho de proyecto. (320-374).</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>Sin urgencia</t>
+          <t>Simple</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
@@ -729,17 +729,17 @@
       </c>
       <c r="G4" s="11" t="inlineStr">
         <is>
-          <t>Ingreso fallo del Tribunal Constitucional</t>
+          <t>Primer informe de comisión Medio Ambiente y Recursos Naturales</t>
         </is>
       </c>
       <c r="H4" s="4" t="inlineStr">
         <is>
-          <t>Miércoles 22 de Abril, 2026</t>
+          <t>10 de enero de 2024</t>
         </is>
       </c>
       <c r="I4" s="11" t="inlineStr">
         <is>
-          <t>Trámite en Tribunal Constitucional / C.Diputados — Oficio</t>
+          <t>Segundo trámite constitucional / C.Diputados — Oficio</t>
         </is>
       </c>
       <c r="J4" s="4" t="inlineStr">
@@ -749,12 +749,12 @@
       </c>
       <c r="K4" s="4" t="inlineStr">
         <is>
-          <t>C.Diputados</t>
+          <t>Senado</t>
         </is>
       </c>
       <c r="L4" s="11" t="inlineStr">
         <is>
-          <t>Ministerio de Hacienda</t>
+          <t>Ministerio de Agricultura; Ministerio de Economía, Fomento y Turismo; Ministerio de Energía; Ministerio de Hacienda; Ministerio de Obras Públicas; Ministerio del Medio Ambiente</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Agrega boletín 18754-17 (reforma INDH)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/seguimiento_legislativo.xlsx
+++ b/seguimiento_legislativo.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Seguimiento Legislativo" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Seguimiento Legislativo" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -496,7 +496,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L16"/>
+  <dimension ref="A1:L17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -575,27 +575,27 @@
     <row r="2" ht="70" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>18216-05</t>
+          <t>18754-17</t>
         </is>
       </c>
       <c r="B2" s="11" t="inlineStr">
         <is>
-          <t>Para la reconstrucción nacional y el desarrollo económico y social</t>
+          <t>Reforma el Instituto Nacional de Derechos Humanos</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>09/10/2026</t>
+          <t>19/10/2026</t>
         </is>
       </c>
       <c r="D2" s="11" t="inlineStr">
         <is>
-          <t>Trámite finalización en Cámara de Origen / C.Diputados — Oficio de ley al Ejecutivo .</t>
+          <t>Primer trámite constitucional / C.Diputados — Cuenta del Mensaje 389-374 que hace presente la urgencia Suma</t>
         </is>
       </c>
       <c r="E2" s="4" t="inlineStr">
         <is>
-          <t>Sin urgencia</t>
+          <t>Suma</t>
         </is>
       </c>
       <c r="F2" s="4" t="inlineStr">
@@ -605,17 +605,17 @@
       </c>
       <c r="G2" s="11" t="inlineStr">
         <is>
-          <t>En espera de promulgación</t>
+          <t>Derechos Humanos y Pueblos Originarios</t>
         </is>
       </c>
       <c r="H2" s="4" t="inlineStr">
         <is>
-          <t>Miércoles 22 de Abril, 2026</t>
+          <t>Lunes 19 de Octubre, 2026</t>
         </is>
       </c>
       <c r="I2" s="11" t="inlineStr">
         <is>
-          <t>Trámite finalización en Cámara de Origen / C.Diputados — Oficio</t>
+          <t>Primer trámite constitucional / C.Diputados</t>
         </is>
       </c>
       <c r="J2" s="4" t="inlineStr">
@@ -630,54 +630,54 @@
       </c>
       <c r="L2" s="11" t="inlineStr">
         <is>
-          <t>Ministerio de Hacienda</t>
+          <t>Ministerio de Justicia y de Derechos Humanos</t>
         </is>
       </c>
     </row>
     <row r="3" ht="70" customHeight="1">
       <c r="A3" s="5" t="inlineStr">
         <is>
-          <t>16553-12</t>
+          <t>18216-05</t>
         </is>
       </c>
       <c r="B3" s="12" t="inlineStr">
         <is>
-          <t>Fortalece y mejora la eficacia de la fiscalización y el cumplimiento de la regulación ambiental a cargo de la Superintendencia del Medio Ambiente, y regula otras materias que indica</t>
+          <t>Para la reconstrucción nacional y el desarrollo económico y social</t>
         </is>
       </c>
       <c r="C3" s="7" t="inlineStr">
         <is>
-          <t>06/10/2026</t>
+          <t>09/10/2026</t>
         </is>
       </c>
       <c r="D3" s="12" t="inlineStr">
         <is>
-          <t>Segundo trámite constitucional / Senado — Cuenta del Mensaje 374-374 que retira y hace presente la urgencia Simple</t>
+          <t>Trámite finalización en Cámara de Origen / C.Diputados — Oficio de ley al Ejecutivo .</t>
         </is>
       </c>
       <c r="E3" s="7" t="inlineStr">
         <is>
-          <t>Simple</t>
+          <t>Sin urgencia</t>
         </is>
       </c>
       <c r="F3" s="7" t="inlineStr">
         <is>
-          <t>Senado</t>
+          <t>Cámara</t>
         </is>
       </c>
       <c r="G3" s="12" t="inlineStr">
         <is>
-          <t>Medio Ambiente, Cambio Climático y Bienes Nacionales</t>
+          <t>En espera de promulgación</t>
         </is>
       </c>
       <c r="H3" s="7" t="inlineStr">
         <is>
-          <t>Miércoles 10 de Enero, 2024</t>
+          <t>Miércoles 22 de Abril, 2026</t>
         </is>
       </c>
       <c r="I3" s="12" t="inlineStr">
         <is>
-          <t>Segundo trámite constitucional / Senado</t>
+          <t>Trámite finalización en Cámara de Origen / C.Diputados — Oficio</t>
         </is>
       </c>
       <c r="J3" s="7" t="inlineStr">
@@ -692,29 +692,29 @@
       </c>
       <c r="L3" s="12" t="inlineStr">
         <is>
-          <t>Ministerio del Medio Ambiente</t>
+          <t>Ministerio de Hacienda</t>
         </is>
       </c>
     </row>
     <row r="4" ht="70" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>16.552-12</t>
+          <t>16553-12</t>
         </is>
       </c>
       <c r="B4" s="11" t="inlineStr">
         <is>
-          <t>Modifica diversos cuerpos legales, con el objeto de fortalecer la institucionalidad ambiental y mejorar su eficiencia</t>
+          <t>Fortalece y mejora la eficacia de la fiscalización y el cumplimiento de la regulación ambiental a cargo de la Superintendencia del Medio Ambiente, y regula otras materias que indica</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>09/09/2026</t>
+          <t>06/10/2026</t>
         </is>
       </c>
       <c r="D4" s="11" t="inlineStr">
         <is>
-          <t>Segundo trámite constitucional / C.Diputados — S.E. el Presidente de la República retira la urgencia "simple", hecha presente para el despacho de proyecto. (320-374).</t>
+          <t>Segundo trámite constitucional / Senado — Cuenta del Mensaje 374-374 que retira y hace presente la urgencia Simple</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
@@ -724,22 +724,22 @@
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>Cámara</t>
+          <t>Senado</t>
         </is>
       </c>
       <c r="G4" s="11" t="inlineStr">
         <is>
-          <t>Primer informe de comisión Medio Ambiente y Recursos Naturales</t>
+          <t>Medio Ambiente, Cambio Climático y Bienes Nacionales</t>
         </is>
       </c>
       <c r="H4" s="4" t="inlineStr">
         <is>
-          <t>10 de enero de 2024</t>
+          <t>Miércoles 10 de Enero, 2024</t>
         </is>
       </c>
       <c r="I4" s="11" t="inlineStr">
         <is>
-          <t>Segundo trámite constitucional / C.Diputados — Oficio</t>
+          <t>Segundo trámite constitucional / Senado</t>
         </is>
       </c>
       <c r="J4" s="4" t="inlineStr">
@@ -749,39 +749,39 @@
       </c>
       <c r="K4" s="4" t="inlineStr">
         <is>
-          <t>Senado</t>
+          <t>C.Diputados</t>
         </is>
       </c>
       <c r="L4" s="11" t="inlineStr">
         <is>
-          <t>Ministerio de Agricultura; Ministerio de Economía, Fomento y Turismo; Ministerio de Energía; Ministerio de Hacienda; Ministerio de Obras Públicas; Ministerio del Medio Ambiente</t>
+          <t>Ministerio del Medio Ambiente</t>
         </is>
       </c>
     </row>
     <row r="5" ht="70" customHeight="1">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>16.075-06</t>
+          <t>16.552-12</t>
         </is>
       </c>
       <c r="B5" s="12" t="inlineStr">
         <is>
-          <t>Modifica cuerpos legales que indica en materia de transparencia e información de fondos recibidos por organizaciones de interés público</t>
+          <t>Modifica diversos cuerpos legales, con el objeto de fortalecer la institucionalidad ambiental y mejorar su eficiencia</t>
         </is>
       </c>
       <c r="C5" s="7" t="inlineStr">
         <is>
-          <t>09/06/2026</t>
+          <t>09/09/2026</t>
         </is>
       </c>
       <c r="D5" s="12" t="inlineStr">
         <is>
-          <t>Primer trámite constitucional / C.Diputados — Archivado. Cuenta oficio N°13/1/2026, de la Comisión de Gobierno Interior, mediante el cual comunica decisión de archivar el proyecto. REMÍTASE AL ARCHIVO</t>
+          <t>Segundo trámite constitucional / C.Diputados — S.E. el Presidente de la República retira la urgencia "simple", hecha presente para el despacho de proyecto. (320-374).</t>
         </is>
       </c>
       <c r="E5" s="7" t="inlineStr">
         <is>
-          <t>Sin urgencia</t>
+          <t>Simple</t>
         </is>
       </c>
       <c r="F5" s="7" t="inlineStr">
@@ -791,44 +791,44 @@
       </c>
       <c r="G5" s="12" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Primer informe de comisión Medio Ambiente y Recursos Naturales</t>
         </is>
       </c>
       <c r="H5" s="7" t="inlineStr">
         <is>
-          <t>4 de julio de 2023</t>
+          <t>10 de enero de 2024</t>
         </is>
       </c>
       <c r="I5" s="12" t="inlineStr">
         <is>
-          <t>Primer trámite constitucional / C.Diputados</t>
+          <t>Segundo trámite constitucional / C.Diputados — Oficio</t>
         </is>
       </c>
       <c r="J5" s="7" t="inlineStr">
         <is>
-          <t>Moción</t>
+          <t>Mensaje</t>
         </is>
       </c>
       <c r="K5" s="7" t="inlineStr">
         <is>
-          <t>Cámara de Diputados</t>
+          <t>Senado</t>
         </is>
       </c>
       <c r="L5" s="12" t="inlineStr">
         <is>
-          <t>Danisa Astudillo Peiretti; Miguel Ángel Calisto Águila; Karol Cariola Oliva; Daniella Cicardini Milla; Marcos Ilabaca Cerda; Daniel Manouchehri Lobos; Vlado Mirosevic Verdugo; Javiera Morales Alvarado; Leonardo Soto Ferrada; Renzo Trisotti Martínez</t>
+          <t>Ministerio de Agricultura; Ministerio de Economía, Fomento y Turismo; Ministerio de Energía; Ministerio de Hacienda; Ministerio de Obras Públicas; Ministerio del Medio Ambiente</t>
         </is>
       </c>
     </row>
     <row r="6" ht="70" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>16.064-06</t>
+          <t>16.075-06</t>
         </is>
       </c>
       <c r="B6" s="11" t="inlineStr">
         <is>
-          <t>Establece una regulación para la conformación y funcionamiento de organizaciones no gubernamentales</t>
+          <t>Modifica cuerpos legales que indica en materia de transparencia e información de fondos recibidos por organizaciones de interés público</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
@@ -858,7 +858,7 @@
       </c>
       <c r="H6" s="4" t="inlineStr">
         <is>
-          <t>3 de julio de 2023</t>
+          <t>4 de julio de 2023</t>
         </is>
       </c>
       <c r="I6" s="11" t="inlineStr">
@@ -878,19 +878,19 @@
       </c>
       <c r="L6" s="11" t="inlineStr">
         <is>
-          <t>Miguel Ángel Calisto Águila; Johannes Kaiser Barents-Von Hohenhagen; Erika Olivera De La Fuente; Joanna Pérez Olea; Jorge Saffirio Espinoza; Carolina Tello Rojas</t>
+          <t>Danisa Astudillo Peiretti; Miguel Ángel Calisto Águila; Karol Cariola Oliva; Daniella Cicardini Milla; Marcos Ilabaca Cerda; Daniel Manouchehri Lobos; Vlado Mirosevic Verdugo; Javiera Morales Alvarado; Leonardo Soto Ferrada; Renzo Trisotti Martínez</t>
         </is>
       </c>
     </row>
     <row r="7" ht="70" customHeight="1">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>16.063-06</t>
+          <t>16.064-06</t>
         </is>
       </c>
       <c r="B7" s="12" t="inlineStr">
         <is>
-          <t>Modifica la ley N° 20.500, sobre asociaciones y participación ciudadana en la gestión pública, para establecer el deber de informar respecto del financiamiento y aportes recibidos de privados</t>
+          <t>Establece una regulación para la conformación y funcionamiento de organizaciones no gubernamentales</t>
         </is>
       </c>
       <c r="C7" s="7" t="inlineStr">
@@ -940,29 +940,29 @@
       </c>
       <c r="L7" s="12" t="inlineStr">
         <is>
-          <t>Jorge Brito Hasbún; Andrés Giordano Salazar; Claudia Mix Jiménez; Javiera Morales Alvarado; Ericka Ñanco Vásquez; Maite Orsini Pascal; Camila Rojas Valderrama; Jaime Sáez Quiroz; Consuelo Veloso Ávila</t>
+          <t>Miguel Ángel Calisto Águila; Johannes Kaiser Barents-Von Hohenhagen; Erika Olivera De La Fuente; Joanna Pérez Olea; Jorge Saffirio Espinoza; Carolina Tello Rojas</t>
         </is>
       </c>
     </row>
     <row r="8" ht="70" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>15.643-06</t>
+          <t>16.063-06</t>
         </is>
       </c>
       <c r="B8" s="11" t="inlineStr">
         <is>
-          <t>Modifica normas legales que indica para obligar a las organizaciones no gubernamentales a transparentar sus ingresos y mecanismos de financiamiento</t>
+          <t>Modifica la ley N° 20.500, sobre asociaciones y participación ciudadana en la gestión pública, para establecer el deber de informar respecto del financiamiento y aportes recibidos de privados</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>02/06/2026</t>
+          <t>09/06/2026</t>
         </is>
       </c>
       <c r="D8" s="11" t="inlineStr">
         <is>
-          <t>Segundo trámite constitucional / Senado — Cuenta del Mensaje 123-374 que retira y hace presente la urgencia Simple</t>
+          <t>Primer trámite constitucional / C.Diputados — Archivado. Cuenta oficio N°13/1/2026, de la Comisión de Gobierno Interior, mediante el cual comunica decisión de archivar el proyecto. REMÍTASE AL ARCHIVO</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
@@ -972,22 +972,22 @@
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>Senado</t>
+          <t>Cámara</t>
         </is>
       </c>
       <c r="G8" s="11" t="inlineStr">
         <is>
-          <t>Gobierno, Descentralización y Regionalización</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H8" s="4" t="inlineStr">
         <is>
-          <t>3 de enero de 2023</t>
+          <t>3 de julio de 2023</t>
         </is>
       </c>
       <c r="I8" s="11" t="inlineStr">
         <is>
-          <t>Segundo trámite constitucional / Senado</t>
+          <t>Primer trámite constitucional / C.Diputados</t>
         </is>
       </c>
       <c r="J8" s="4" t="inlineStr">
@@ -1002,19 +1002,19 @@
       </c>
       <c r="L8" s="11" t="inlineStr">
         <is>
-          <t>Miguel Ángel Calisto Águila; Erika Olivera De La Fuente; Joanna Pérez Olea; Jorge Saffirio Espinoza; Leonardo Soto Ferrada</t>
+          <t>Jorge Brito Hasbún; Andrés Giordano Salazar; Claudia Mix Jiménez; Javiera Morales Alvarado; Ericka Ñanco Vásquez; Maite Orsini Pascal; Camila Rojas Valderrama; Jaime Sáez Quiroz; Consuelo Veloso Ávila</t>
         </is>
       </c>
     </row>
     <row r="9" ht="70" customHeight="1">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>17.817-07</t>
+          <t>15.643-06</t>
         </is>
       </c>
       <c r="B9" s="12" t="inlineStr">
         <is>
-          <t>Moderniza el régimen normativo de las corporaciones y fundaciones, y fortalece su fiscalización</t>
+          <t>Modifica normas legales que indica para obligar a las organizaciones no gubernamentales a transparentar sus ingresos y mecanismos de financiamiento</t>
         </is>
       </c>
       <c r="C9" s="7" t="inlineStr">
@@ -1024,37 +1024,37 @@
       </c>
       <c r="D9" s="12" t="inlineStr">
         <is>
-          <t>Primer trámite constitucional / C.Diputados — Cuenta del Mensaje 122-374 que hace presente la urgencia Simple</t>
+          <t>Segundo trámite constitucional / Senado — Cuenta del Mensaje 123-374 que retira y hace presente la urgencia Simple</t>
         </is>
       </c>
       <c r="E9" s="7" t="inlineStr">
         <is>
-          <t>Simple</t>
+          <t>Sin urgencia</t>
         </is>
       </c>
       <c r="F9" s="7" t="inlineStr">
         <is>
-          <t>Cámara</t>
+          <t>Senado</t>
         </is>
       </c>
       <c r="G9" s="12" t="inlineStr">
         <is>
-          <t>Constitución, Legislación, Justicia y Reglamento</t>
+          <t>Gobierno, Descentralización y Regionalización</t>
         </is>
       </c>
       <c r="H9" s="7" t="inlineStr">
         <is>
-          <t>8 de septiembre de 2025</t>
+          <t>3 de enero de 2023</t>
         </is>
       </c>
       <c r="I9" s="12" t="inlineStr">
         <is>
-          <t>Primer trámite constitucional / C.Diputados</t>
+          <t>Segundo trámite constitucional / Senado</t>
         </is>
       </c>
       <c r="J9" s="7" t="inlineStr">
         <is>
-          <t>Mensaje</t>
+          <t>Moción</t>
         </is>
       </c>
       <c r="K9" s="7" t="inlineStr">
@@ -1064,29 +1064,29 @@
       </c>
       <c r="L9" s="12" t="inlineStr">
         <is>
-          <t>Ministerio de Justicia y Derechos Humanos</t>
+          <t>Miguel Ángel Calisto Águila; Erika Olivera De La Fuente; Joanna Pérez Olea; Jorge Saffirio Espinoza; Leonardo Soto Ferrada</t>
         </is>
       </c>
     </row>
     <row r="10" ht="70" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>16.888-06</t>
+          <t>17.817-07</t>
         </is>
       </c>
       <c r="B10" s="11" t="inlineStr">
         <is>
-          <t>Moderniza la regulación del lobby y las gestiones de intereses particulares ante las autoridades y funcionarios</t>
+          <t>Moderniza el régimen normativo de las corporaciones y fundaciones, y fortalece su fiscalización</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>13/05/2026</t>
+          <t>02/06/2026</t>
         </is>
       </c>
       <c r="D10" s="11" t="inlineStr">
         <is>
-          <t>Primer trámite constitucional / C.Diputados — Discusión general . Queda pendiente</t>
+          <t>Primer trámite constitucional / C.Diputados — Cuenta del Mensaje 122-374 que hace presente la urgencia Simple</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
@@ -1101,17 +1101,17 @@
       </c>
       <c r="G10" s="11" t="inlineStr">
         <is>
-          <t>En Sala</t>
+          <t>Constitución, Legislación, Justicia y Reglamento</t>
         </is>
       </c>
       <c r="H10" s="4" t="inlineStr">
         <is>
-          <t>31 de mayo de 2024</t>
+          <t>8 de septiembre de 2025</t>
         </is>
       </c>
       <c r="I10" s="11" t="inlineStr">
         <is>
-          <t>Primer trámite constitucional / C.Diputados — Diario</t>
+          <t>Primer trámite constitucional / C.Diputados</t>
         </is>
       </c>
       <c r="J10" s="4" t="inlineStr">
@@ -1126,29 +1126,29 @@
       </c>
       <c r="L10" s="11" t="inlineStr">
         <is>
-          <t>Ministerio Secretaría General de Gobierno; Ministerio Secretaría General de la Presidencia; Ministerio de Hacienda; Ministerio de Justicia y Derechos Humanos</t>
+          <t>Ministerio de Justicia y Derechos Humanos</t>
         </is>
       </c>
     </row>
     <row r="11" ht="70" customHeight="1">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>16746-06</t>
+          <t>16.888-06</t>
         </is>
       </c>
       <c r="B11" s="12" t="inlineStr">
         <is>
-          <t>Modifica la ley N° 20.285, sobre acceso a la informacion pública, para elevar los estándares de transparencia corporativa exigible a las empresas públicas</t>
+          <t>Moderniza la regulación del lobby y las gestiones de intereses particulares ante las autoridades y funcionarios</t>
         </is>
       </c>
       <c r="C11" s="7" t="inlineStr">
         <is>
-          <t>23/03/2026</t>
+          <t>13/05/2026</t>
         </is>
       </c>
       <c r="D11" s="12" t="inlineStr">
         <is>
-          <t>Primer trámite constitucional / C.Diputados — Cuenta del Mensaje 14-374 que hace presente la urgencia Simple</t>
+          <t>Primer trámite constitucional / C.Diputados — Discusión general . Queda pendiente</t>
         </is>
       </c>
       <c r="E11" s="7" t="inlineStr">
@@ -1163,59 +1163,59 @@
       </c>
       <c r="G11" s="12" t="inlineStr">
         <is>
-          <t>Gobierno Interior Nacionalidad Ciudadanía y Regionalización</t>
+          <t>En Sala</t>
         </is>
       </c>
       <c r="H11" s="7" t="inlineStr">
         <is>
-          <t>Miércoles 10 de Abril, 2024</t>
+          <t>31 de mayo de 2024</t>
         </is>
       </c>
       <c r="I11" s="12" t="inlineStr">
         <is>
-          <t>Primer trámite constitucional / C.Diputados</t>
+          <t>Primer trámite constitucional / C.Diputados — Diario</t>
         </is>
       </c>
       <c r="J11" s="7" t="inlineStr">
         <is>
-          <t>Moción</t>
+          <t>Mensaje</t>
         </is>
       </c>
       <c r="K11" s="7" t="inlineStr">
         <is>
-          <t>C.Diputados</t>
+          <t>Cámara de Diputados</t>
         </is>
       </c>
       <c r="L11" s="12" t="inlineStr">
         <is>
-          <t>Becker Alvear, Miguel Ángel; Berger Fett, Bernardo; Castro Bascuñán, José Miguel; Fuenzalida Cobo, Juan; Jouannet Valderrama, Andrés; Matheson Villán, Christian; Meza Pereira, José Carlos; Tapia Ramos, Cristián; Weisse Novoa, Flor</t>
+          <t>Ministerio Secretaría General de Gobierno; Ministerio Secretaría General de la Presidencia; Ministerio de Hacienda; Ministerio de Justicia y Derechos Humanos</t>
         </is>
       </c>
     </row>
     <row r="12" ht="70" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>17.797-06</t>
+          <t>16746-06</t>
         </is>
       </c>
       <c r="B12" s="11" t="inlineStr">
         <is>
-          <t>Modifica la ley N° 20.500, sobre Asociaciones y Participación Ciudadana en la Gestión Pública, y otros cuerpos normativos que indica</t>
+          <t>Modifica la ley N° 20.285, sobre acceso a la informacion pública, para elevar los estándares de transparencia corporativa exigible a las empresas públicas</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>02/03/2026</t>
+          <t>23/03/2026</t>
         </is>
       </c>
       <c r="D12" s="11" t="inlineStr">
         <is>
-          <t>Primer trámite constitucional / C.Diputados — Cuenta del Mensaje 1602-373 que hace presente la urgencia Suma</t>
+          <t>Primer trámite constitucional / C.Diputados — Cuenta del Mensaje 14-374 que hace presente la urgencia Simple</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>Suma</t>
+          <t>Simple</t>
         </is>
       </c>
       <c r="F12" s="4" t="inlineStr">
@@ -1230,7 +1230,7 @@
       </c>
       <c r="H12" s="4" t="inlineStr">
         <is>
-          <t>1 de septiembre de 2025</t>
+          <t>Miércoles 10 de Abril, 2024</t>
         </is>
       </c>
       <c r="I12" s="11" t="inlineStr">
@@ -1240,69 +1240,69 @@
       </c>
       <c r="J12" s="4" t="inlineStr">
         <is>
-          <t>Mensaje</t>
+          <t>Moción</t>
         </is>
       </c>
       <c r="K12" s="4" t="inlineStr">
         <is>
-          <t>Cámara de Diputados</t>
+          <t>C.Diputados</t>
         </is>
       </c>
       <c r="L12" s="11" t="inlineStr">
         <is>
-          <t>Ministerio Secretaría General de Gobierno</t>
+          <t>Becker Alvear, Miguel Ángel; Berger Fett, Bernardo; Castro Bascuñán, José Miguel; Fuenzalida Cobo, Juan; Jouannet Valderrama, Andrés; Matheson Villán, Christian; Meza Pereira, José Carlos; Tapia Ramos, Cristián; Weisse Novoa, Flor</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>16.886-12</t>
+          <t>17.797-06</t>
         </is>
       </c>
       <c r="B13" s="12" t="inlineStr">
         <is>
-          <t>Dicta normas sobre protección de personas defensoras de la naturaleza y los derechos humanos medioambientales</t>
+          <t>Modifica la ley N° 20.500, sobre Asociaciones y Participación Ciudadana en la Gestión Pública, y otros cuerpos normativos que indica</t>
         </is>
       </c>
       <c r="C13" s="7" t="inlineStr">
         <is>
-          <t>08/10/2025</t>
+          <t>02/03/2026</t>
         </is>
       </c>
       <c r="D13" s="12" t="inlineStr">
         <is>
-          <t>Segundo trámite constitucional / Senado — Cuenta de proyecto . Pasa a Comisión de Derechos Humanos, Nacionalidad y Ciudadanía</t>
+          <t>Primer trámite constitucional / C.Diputados — Cuenta del Mensaje 1602-373 que hace presente la urgencia Suma</t>
         </is>
       </c>
       <c r="E13" s="7" t="inlineStr">
         <is>
-          <t>Sin urgencia</t>
+          <t>Suma</t>
         </is>
       </c>
       <c r="F13" s="7" t="inlineStr">
         <is>
-          <t>Senado</t>
+          <t>Cámara</t>
         </is>
       </c>
       <c r="G13" s="12" t="inlineStr">
         <is>
-          <t>Derechos Humanos, Nacionalidad y Ciudadanía</t>
+          <t>Gobierno Interior Nacionalidad Ciudadanía y Regionalización</t>
         </is>
       </c>
       <c r="H13" s="7" t="inlineStr">
         <is>
-          <t>29 de mayo de 2024</t>
+          <t>1 de septiembre de 2025</t>
         </is>
       </c>
       <c r="I13" s="12" t="inlineStr">
         <is>
-          <t>Segundo trámite constitucional / Senado</t>
+          <t>Primer trámite constitucional / C.Diputados</t>
         </is>
       </c>
       <c r="J13" s="7" t="inlineStr">
         <is>
-          <t>Moción</t>
+          <t>Mensaje</t>
         </is>
       </c>
       <c r="K13" s="7" t="inlineStr">
@@ -1312,29 +1312,29 @@
       </c>
       <c r="L13" s="12" t="inlineStr">
         <is>
-          <t>Alejandro Bernales; Viviana Delgado; Luis Malla (A); Vlado Mirosevic; Sebastián Videla</t>
+          <t>Ministerio Secretaría General de Gobierno</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>17.520-17</t>
+          <t>16.886-12</t>
         </is>
       </c>
       <c r="B14" s="11" t="inlineStr">
         <is>
-          <t>Establece la obligación de incorporar la debida diligencia en derechos humanos a las empresas que operen en territorio nacional</t>
+          <t>Dicta normas sobre protección de personas defensoras de la naturaleza y los derechos humanos medioambientales</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>07/05/2025</t>
+          <t>08/10/2025</t>
         </is>
       </c>
       <c r="D14" s="11" t="inlineStr">
         <is>
-          <t>Primer trámite constitucional / C.Diputados — Oficio N° 20406. Deriva a la Comisión de Economía, Fomento; Micro, Pequeña y Mediana Empresa; Protección de los Consumidores y Turismo, el proyecto de ley asignado inicialmente a la Comisión de Derechos Humanos.</t>
+          <t>Segundo trámite constitucional / Senado — Cuenta de proyecto . Pasa a Comisión de Derechos Humanos, Nacionalidad y Ciudadanía</t>
         </is>
       </c>
       <c r="E14" s="4" t="inlineStr">
@@ -1344,22 +1344,22 @@
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>Cámara</t>
+          <t>Senado</t>
         </is>
       </c>
       <c r="G14" s="11" t="inlineStr">
         <is>
-          <t>Derechos Humanos y Pueblos Originarios</t>
+          <t>Derechos Humanos, Nacionalidad y Ciudadanía</t>
         </is>
       </c>
       <c r="H14" s="4" t="inlineStr">
         <is>
-          <t>5 de mayo de 2025</t>
+          <t>29 de mayo de 2024</t>
         </is>
       </c>
       <c r="I14" s="11" t="inlineStr">
         <is>
-          <t>Primer trámite constitucional / C.Diputados — Oficio</t>
+          <t>Segundo trámite constitucional / Senado</t>
         </is>
       </c>
       <c r="J14" s="4" t="inlineStr">
@@ -1374,29 +1374,29 @@
       </c>
       <c r="L14" s="11" t="inlineStr">
         <is>
-          <t>María Francisca Bello Campos; Roberto Celedón Fernández; Lorena Fries Monleón; Andrés Giordano Salazar; Diego Ibáñez Cotroneo; Camila Rojas Valderrama; Jaime Sáez Quiroz; Clara Sagardia Cabezas; Carolina Tello Rojas; Gael Yeomans Araya</t>
+          <t>Alejandro Bernales; Viviana Delgado; Luis Malla (A); Vlado Mirosevic; Sebastián Videla</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>17.446-17</t>
+          <t>17.520-17</t>
         </is>
       </c>
       <c r="B15" s="12" t="inlineStr">
         <is>
-          <t>Establece y regula la debida diligencia de las empresas en el respeto a los derechos humanos, el medio ambiente y el cambio climático</t>
+          <t>Establece la obligación de incorporar la debida diligencia en derechos humanos a las empresas que operen en territorio nacional</t>
         </is>
       </c>
       <c r="C15" s="7" t="inlineStr">
         <is>
-          <t>08/04/2025</t>
+          <t>07/05/2025</t>
         </is>
       </c>
       <c r="D15" s="12" t="inlineStr">
         <is>
-          <t>Primer trámite constitucional / Senado — Cuenta de proyecto . Pasa a Comisión de Derechos Humanos, Nacionalidad y Ciudadanía</t>
+          <t>Primer trámite constitucional / C.Diputados — Oficio N° 20406. Deriva a la Comisión de Economía, Fomento; Micro, Pequeña y Mediana Empresa; Protección de los Consumidores y Turismo, el proyecto de ley asignado inicialmente a la Comisión de Derechos Humanos.</t>
         </is>
       </c>
       <c r="E15" s="7" t="inlineStr">
@@ -1406,22 +1406,22 @@
       </c>
       <c r="F15" s="7" t="inlineStr">
         <is>
-          <t>Senado</t>
+          <t>Cámara</t>
         </is>
       </c>
       <c r="G15" s="12" t="inlineStr">
         <is>
-          <t>Derechos Humanos, Nacionalidad y Ciudadanía</t>
+          <t>Derechos Humanos y Pueblos Originarios</t>
         </is>
       </c>
       <c r="H15" s="7" t="inlineStr">
         <is>
-          <t>3 de abril de 2025</t>
+          <t>5 de mayo de 2025</t>
         </is>
       </c>
       <c r="I15" s="12" t="inlineStr">
         <is>
-          <t>Primer trámite constitucional / Senado</t>
+          <t>Primer trámite constitucional / C.Diputados — Oficio</t>
         </is>
       </c>
       <c r="J15" s="7" t="inlineStr">
@@ -1431,72 +1431,134 @@
       </c>
       <c r="K15" s="7" t="inlineStr">
         <is>
-          <t>Senado</t>
+          <t>Cámara de Diputados</t>
         </is>
       </c>
       <c r="L15" s="12" t="inlineStr">
         <is>
-          <t>Isabel Allende Bussi</t>
+          <t>María Francisca Bello Campos; Roberto Celedón Fernández; Lorena Fries Monleón; Andrés Giordano Salazar; Diego Ibáñez Cotroneo; Camila Rojas Valderrama; Jaime Sáez Quiroz; Clara Sagardia Cabezas; Carolina Tello Rojas; Gael Yeomans Araya</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
+          <t>17.446-17</t>
+        </is>
+      </c>
+      <c r="B16" s="11" t="inlineStr">
+        <is>
+          <t>Establece y regula la debida diligencia de las empresas en el respeto a los derechos humanos, el medio ambiente y el cambio climático</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>08/04/2025</t>
+        </is>
+      </c>
+      <c r="D16" s="11" t="inlineStr">
+        <is>
+          <t>Primer trámite constitucional / Senado — Cuenta de proyecto . Pasa a Comisión de Derechos Humanos, Nacionalidad y Ciudadanía</t>
+        </is>
+      </c>
+      <c r="E16" s="4" t="inlineStr">
+        <is>
+          <t>Sin urgencia</t>
+        </is>
+      </c>
+      <c r="F16" s="4" t="inlineStr">
+        <is>
+          <t>Senado</t>
+        </is>
+      </c>
+      <c r="G16" s="11" t="inlineStr">
+        <is>
+          <t>Derechos Humanos, Nacionalidad y Ciudadanía</t>
+        </is>
+      </c>
+      <c r="H16" s="4" t="inlineStr">
+        <is>
+          <t>3 de abril de 2025</t>
+        </is>
+      </c>
+      <c r="I16" s="11" t="inlineStr">
+        <is>
+          <t>Primer trámite constitucional / Senado</t>
+        </is>
+      </c>
+      <c r="J16" s="4" t="inlineStr">
+        <is>
+          <t>Moción</t>
+        </is>
+      </c>
+      <c r="K16" s="4" t="inlineStr">
+        <is>
+          <t>Senado</t>
+        </is>
+      </c>
+      <c r="L16" s="11" t="inlineStr">
+        <is>
+          <t>Isabel Allende Bussi</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
           <t>17196-17</t>
         </is>
       </c>
-      <c r="B16" s="11" t="inlineStr">
+      <c r="B17" s="12" t="inlineStr">
         <is>
           <t>Modifica la ley N° 18.046, Ley sobre Sociedades Anónimas, con el objeto de establecer obligaciones para promover la protección de derechos humanos, a las personas jurídicas que indica.</t>
         </is>
       </c>
-      <c r="C16" s="4" t="inlineStr">
+      <c r="C17" s="7" t="inlineStr">
         <is>
           <t>21/10/2024</t>
         </is>
       </c>
-      <c r="D16" s="11" t="inlineStr">
+      <c r="D17" s="12" t="inlineStr">
         <is>
           <t>Primer trámite constitucional / Senado — Cuenta de proyecto . Pasa a Comisión de Derechos Humanos, Nacionalidad y Ciudadanía</t>
         </is>
       </c>
-      <c r="E16" s="4" t="inlineStr">
+      <c r="E17" s="7" t="inlineStr">
         <is>
           <t>Sin urgencia</t>
         </is>
       </c>
-      <c r="F16" s="4" t="inlineStr">
+      <c r="F17" s="7" t="inlineStr">
         <is>
           <t>Senado</t>
         </is>
       </c>
-      <c r="G16" s="11" t="inlineStr">
+      <c r="G17" s="12" t="inlineStr">
         <is>
           <t>Derechos Humanos, Nacionalidad y Ciudadanía</t>
         </is>
       </c>
-      <c r="H16" s="4" t="inlineStr">
+      <c r="H17" s="7" t="inlineStr">
         <is>
           <t>Lunes 21 de Octubre, 2024</t>
         </is>
       </c>
-      <c r="I16" s="11" t="inlineStr">
+      <c r="I17" s="12" t="inlineStr">
         <is>
           <t>Primer trámite constitucional / Senado</t>
         </is>
       </c>
-      <c r="J16" s="4" t="inlineStr">
+      <c r="J17" s="7" t="inlineStr">
         <is>
           <t>Moción</t>
         </is>
       </c>
-      <c r="K16" s="4" t="inlineStr">
+      <c r="K17" s="7" t="inlineStr">
         <is>
           <t>Senado</t>
         </is>
       </c>
-      <c r="L16" s="11" t="inlineStr">
+      <c r="L17" s="12" t="inlineStr">
         <is>
           <t>Vodanovic Rojas, Paulina</t>
         </is>
@@ -1519,6 +1581,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A14" r:id="rId13"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A15" r:id="rId14"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A16" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A17" r:id="rId16"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Agrega boletín 18271-07 (aportes del extranjero a personas jurídicas sin fines de lucro)
</commit_message>
<xml_diff>
--- a/seguimiento_legislativo.xlsx
+++ b/seguimiento_legislativo.xlsx
@@ -496,7 +496,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L17"/>
+  <dimension ref="A1:L18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -637,27 +637,27 @@
     <row r="3" ht="70" customHeight="1">
       <c r="A3" s="5" t="inlineStr">
         <is>
-          <t>18216-05</t>
+          <t>18271-07</t>
         </is>
       </c>
       <c r="B3" s="12" t="inlineStr">
         <is>
-          <t>Para la reconstrucción nacional y el desarrollo económico y social</t>
+          <t>Establece la obligación de declarar los aportes provenientes desde el extranjero para personas jurídicas sin fines de lucro</t>
         </is>
       </c>
       <c r="C3" s="7" t="inlineStr">
         <is>
-          <t>09/10/2026</t>
+          <t>19/10/2026</t>
         </is>
       </c>
       <c r="D3" s="12" t="inlineStr">
         <is>
-          <t>Trámite finalización en Cámara de Origen / C.Diputados — Oficio de ley al Ejecutivo .</t>
+          <t>Primer trámite constitucional / C.Diputados — Cuenta del Mensaje 388-374 que retira y hace presente la urgencia Simple</t>
         </is>
       </c>
       <c r="E3" s="7" t="inlineStr">
         <is>
-          <t>Sin urgencia</t>
+          <t>Simple</t>
         </is>
       </c>
       <c r="F3" s="7" t="inlineStr">
@@ -667,22 +667,22 @@
       </c>
       <c r="G3" s="12" t="inlineStr">
         <is>
-          <t>En espera de promulgación</t>
+          <t>Constitución, Legislación, Justicia y Reglamento</t>
         </is>
       </c>
       <c r="H3" s="7" t="inlineStr">
         <is>
-          <t>Miércoles 22 de Abril, 2026</t>
+          <t>Miércoles 13 de Mayo, 2026</t>
         </is>
       </c>
       <c r="I3" s="12" t="inlineStr">
         <is>
-          <t>Trámite finalización en Cámara de Origen / C.Diputados — Oficio</t>
+          <t>Primer trámite constitucional / C.Diputados</t>
         </is>
       </c>
       <c r="J3" s="7" t="inlineStr">
         <is>
-          <t>Mensaje</t>
+          <t>Moción</t>
         </is>
       </c>
       <c r="K3" s="7" t="inlineStr">
@@ -692,54 +692,54 @@
       </c>
       <c r="L3" s="12" t="inlineStr">
         <is>
-          <t>Ministerio de Hacienda</t>
+          <t>Araya  Guerrero, Jaime; Barchiesi  Chávez, Chiara; Kunstmann Collado, Leandro; Malla Valenzuela, Luis; Muñoz Minte, Paulina; Neumann Bertín, Ricardo; Pardo Sáinz, Luis; Ramírez Ramírez, Tamara; Ramírez Diez, Guillermo</t>
         </is>
       </c>
     </row>
     <row r="4" ht="70" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>16553-12</t>
+          <t>18216-05</t>
         </is>
       </c>
       <c r="B4" s="11" t="inlineStr">
         <is>
-          <t>Fortalece y mejora la eficacia de la fiscalización y el cumplimiento de la regulación ambiental a cargo de la Superintendencia del Medio Ambiente, y regula otras materias que indica</t>
+          <t>Para la reconstrucción nacional y el desarrollo económico y social</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>06/10/2026</t>
+          <t>09/10/2026</t>
         </is>
       </c>
       <c r="D4" s="11" t="inlineStr">
         <is>
-          <t>Segundo trámite constitucional / Senado — Cuenta del Mensaje 374-374 que retira y hace presente la urgencia Simple</t>
+          <t>Trámite finalización en Cámara de Origen / C.Diputados — Oficio de ley al Ejecutivo .</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>Simple</t>
+          <t>Sin urgencia</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>Senado</t>
+          <t>Cámara</t>
         </is>
       </c>
       <c r="G4" s="11" t="inlineStr">
         <is>
-          <t>Medio Ambiente, Cambio Climático y Bienes Nacionales</t>
+          <t>En espera de promulgación</t>
         </is>
       </c>
       <c r="H4" s="4" t="inlineStr">
         <is>
-          <t>Miércoles 10 de Enero, 2024</t>
+          <t>Miércoles 22 de Abril, 2026</t>
         </is>
       </c>
       <c r="I4" s="11" t="inlineStr">
         <is>
-          <t>Segundo trámite constitucional / Senado</t>
+          <t>Trámite finalización en Cámara de Origen / C.Diputados — Oficio</t>
         </is>
       </c>
       <c r="J4" s="4" t="inlineStr">
@@ -754,29 +754,29 @@
       </c>
       <c r="L4" s="11" t="inlineStr">
         <is>
-          <t>Ministerio del Medio Ambiente</t>
+          <t>Ministerio de Hacienda</t>
         </is>
       </c>
     </row>
     <row r="5" ht="70" customHeight="1">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>16.552-12</t>
+          <t>16553-12</t>
         </is>
       </c>
       <c r="B5" s="12" t="inlineStr">
         <is>
-          <t>Modifica diversos cuerpos legales, con el objeto de fortalecer la institucionalidad ambiental y mejorar su eficiencia</t>
+          <t>Fortalece y mejora la eficacia de la fiscalización y el cumplimiento de la regulación ambiental a cargo de la Superintendencia del Medio Ambiente, y regula otras materias que indica</t>
         </is>
       </c>
       <c r="C5" s="7" t="inlineStr">
         <is>
-          <t>09/09/2026</t>
+          <t>06/10/2026</t>
         </is>
       </c>
       <c r="D5" s="12" t="inlineStr">
         <is>
-          <t>Segundo trámite constitucional / C.Diputados — S.E. el Presidente de la República retira la urgencia "simple", hecha presente para el despacho de proyecto. (320-374).</t>
+          <t>Segundo trámite constitucional / Senado — Cuenta del Mensaje 374-374 que retira y hace presente la urgencia Simple</t>
         </is>
       </c>
       <c r="E5" s="7" t="inlineStr">
@@ -786,22 +786,22 @@
       </c>
       <c r="F5" s="7" t="inlineStr">
         <is>
-          <t>Cámara</t>
+          <t>Senado</t>
         </is>
       </c>
       <c r="G5" s="12" t="inlineStr">
         <is>
-          <t>Primer informe de comisión Medio Ambiente y Recursos Naturales</t>
+          <t>Medio Ambiente, Cambio Climático y Bienes Nacionales</t>
         </is>
       </c>
       <c r="H5" s="7" t="inlineStr">
         <is>
-          <t>10 de enero de 2024</t>
+          <t>Miércoles 10 de Enero, 2024</t>
         </is>
       </c>
       <c r="I5" s="12" t="inlineStr">
         <is>
-          <t>Segundo trámite constitucional / C.Diputados — Oficio</t>
+          <t>Segundo trámite constitucional / Senado</t>
         </is>
       </c>
       <c r="J5" s="7" t="inlineStr">
@@ -811,39 +811,39 @@
       </c>
       <c r="K5" s="7" t="inlineStr">
         <is>
-          <t>Senado</t>
+          <t>C.Diputados</t>
         </is>
       </c>
       <c r="L5" s="12" t="inlineStr">
         <is>
-          <t>Ministerio de Agricultura; Ministerio de Economía, Fomento y Turismo; Ministerio de Energía; Ministerio de Hacienda; Ministerio de Obras Públicas; Ministerio del Medio Ambiente</t>
+          <t>Ministerio del Medio Ambiente</t>
         </is>
       </c>
     </row>
     <row r="6" ht="70" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>16.075-06</t>
+          <t>16.552-12</t>
         </is>
       </c>
       <c r="B6" s="11" t="inlineStr">
         <is>
-          <t>Modifica cuerpos legales que indica en materia de transparencia e información de fondos recibidos por organizaciones de interés público</t>
+          <t>Modifica diversos cuerpos legales, con el objeto de fortalecer la institucionalidad ambiental y mejorar su eficiencia</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>09/06/2026</t>
+          <t>09/09/2026</t>
         </is>
       </c>
       <c r="D6" s="11" t="inlineStr">
         <is>
-          <t>Primer trámite constitucional / C.Diputados — Archivado. Cuenta oficio N°13/1/2026, de la Comisión de Gobierno Interior, mediante el cual comunica decisión de archivar el proyecto. REMÍTASE AL ARCHIVO</t>
+          <t>Segundo trámite constitucional / C.Diputados — S.E. el Presidente de la República retira la urgencia "simple", hecha presente para el despacho de proyecto. (320-374).</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>Sin urgencia</t>
+          <t>Simple</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr">
@@ -853,44 +853,44 @@
       </c>
       <c r="G6" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Primer informe de comisión Medio Ambiente y Recursos Naturales</t>
         </is>
       </c>
       <c r="H6" s="4" t="inlineStr">
         <is>
-          <t>4 de julio de 2023</t>
+          <t>10 de enero de 2024</t>
         </is>
       </c>
       <c r="I6" s="11" t="inlineStr">
         <is>
-          <t>Primer trámite constitucional / C.Diputados</t>
+          <t>Segundo trámite constitucional / C.Diputados — Oficio</t>
         </is>
       </c>
       <c r="J6" s="4" t="inlineStr">
         <is>
-          <t>Moción</t>
+          <t>Mensaje</t>
         </is>
       </c>
       <c r="K6" s="4" t="inlineStr">
         <is>
-          <t>Cámara de Diputados</t>
+          <t>Senado</t>
         </is>
       </c>
       <c r="L6" s="11" t="inlineStr">
         <is>
-          <t>Danisa Astudillo Peiretti; Miguel Ángel Calisto Águila; Karol Cariola Oliva; Daniella Cicardini Milla; Marcos Ilabaca Cerda; Daniel Manouchehri Lobos; Vlado Mirosevic Verdugo; Javiera Morales Alvarado; Leonardo Soto Ferrada; Renzo Trisotti Martínez</t>
+          <t>Ministerio de Agricultura; Ministerio de Economía, Fomento y Turismo; Ministerio de Energía; Ministerio de Hacienda; Ministerio de Obras Públicas; Ministerio del Medio Ambiente</t>
         </is>
       </c>
     </row>
     <row r="7" ht="70" customHeight="1">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>16.064-06</t>
+          <t>16.075-06</t>
         </is>
       </c>
       <c r="B7" s="12" t="inlineStr">
         <is>
-          <t>Establece una regulación para la conformación y funcionamiento de organizaciones no gubernamentales</t>
+          <t>Modifica cuerpos legales que indica en materia de transparencia e información de fondos recibidos por organizaciones de interés público</t>
         </is>
       </c>
       <c r="C7" s="7" t="inlineStr">
@@ -920,7 +920,7 @@
       </c>
       <c r="H7" s="7" t="inlineStr">
         <is>
-          <t>3 de julio de 2023</t>
+          <t>4 de julio de 2023</t>
         </is>
       </c>
       <c r="I7" s="12" t="inlineStr">
@@ -940,19 +940,19 @@
       </c>
       <c r="L7" s="12" t="inlineStr">
         <is>
-          <t>Miguel Ángel Calisto Águila; Johannes Kaiser Barents-Von Hohenhagen; Erika Olivera De La Fuente; Joanna Pérez Olea; Jorge Saffirio Espinoza; Carolina Tello Rojas</t>
+          <t>Danisa Astudillo Peiretti; Miguel Ángel Calisto Águila; Karol Cariola Oliva; Daniella Cicardini Milla; Marcos Ilabaca Cerda; Daniel Manouchehri Lobos; Vlado Mirosevic Verdugo; Javiera Morales Alvarado; Leonardo Soto Ferrada; Renzo Trisotti Martínez</t>
         </is>
       </c>
     </row>
     <row r="8" ht="70" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>16.063-06</t>
+          <t>16.064-06</t>
         </is>
       </c>
       <c r="B8" s="11" t="inlineStr">
         <is>
-          <t>Modifica la ley N° 20.500, sobre asociaciones y participación ciudadana en la gestión pública, para establecer el deber de informar respecto del financiamiento y aportes recibidos de privados</t>
+          <t>Establece una regulación para la conformación y funcionamiento de organizaciones no gubernamentales</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
@@ -1002,29 +1002,29 @@
       </c>
       <c r="L8" s="11" t="inlineStr">
         <is>
-          <t>Jorge Brito Hasbún; Andrés Giordano Salazar; Claudia Mix Jiménez; Javiera Morales Alvarado; Ericka Ñanco Vásquez; Maite Orsini Pascal; Camila Rojas Valderrama; Jaime Sáez Quiroz; Consuelo Veloso Ávila</t>
+          <t>Miguel Ángel Calisto Águila; Johannes Kaiser Barents-Von Hohenhagen; Erika Olivera De La Fuente; Joanna Pérez Olea; Jorge Saffirio Espinoza; Carolina Tello Rojas</t>
         </is>
       </c>
     </row>
     <row r="9" ht="70" customHeight="1">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>15.643-06</t>
+          <t>16.063-06</t>
         </is>
       </c>
       <c r="B9" s="12" t="inlineStr">
         <is>
-          <t>Modifica normas legales que indica para obligar a las organizaciones no gubernamentales a transparentar sus ingresos y mecanismos de financiamiento</t>
+          <t>Modifica la ley N° 20.500, sobre asociaciones y participación ciudadana en la gestión pública, para establecer el deber de informar respecto del financiamiento y aportes recibidos de privados</t>
         </is>
       </c>
       <c r="C9" s="7" t="inlineStr">
         <is>
-          <t>02/06/2026</t>
+          <t>09/06/2026</t>
         </is>
       </c>
       <c r="D9" s="12" t="inlineStr">
         <is>
-          <t>Segundo trámite constitucional / Senado — Cuenta del Mensaje 123-374 que retira y hace presente la urgencia Simple</t>
+          <t>Primer trámite constitucional / C.Diputados — Archivado. Cuenta oficio N°13/1/2026, de la Comisión de Gobierno Interior, mediante el cual comunica decisión de archivar el proyecto. REMÍTASE AL ARCHIVO</t>
         </is>
       </c>
       <c r="E9" s="7" t="inlineStr">
@@ -1034,22 +1034,22 @@
       </c>
       <c r="F9" s="7" t="inlineStr">
         <is>
-          <t>Senado</t>
+          <t>Cámara</t>
         </is>
       </c>
       <c r="G9" s="12" t="inlineStr">
         <is>
-          <t>Gobierno, Descentralización y Regionalización</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H9" s="7" t="inlineStr">
         <is>
-          <t>3 de enero de 2023</t>
+          <t>3 de julio de 2023</t>
         </is>
       </c>
       <c r="I9" s="12" t="inlineStr">
         <is>
-          <t>Segundo trámite constitucional / Senado</t>
+          <t>Primer trámite constitucional / C.Diputados</t>
         </is>
       </c>
       <c r="J9" s="7" t="inlineStr">
@@ -1064,19 +1064,19 @@
       </c>
       <c r="L9" s="12" t="inlineStr">
         <is>
-          <t>Miguel Ángel Calisto Águila; Erika Olivera De La Fuente; Joanna Pérez Olea; Jorge Saffirio Espinoza; Leonardo Soto Ferrada</t>
+          <t>Jorge Brito Hasbún; Andrés Giordano Salazar; Claudia Mix Jiménez; Javiera Morales Alvarado; Ericka Ñanco Vásquez; Maite Orsini Pascal; Camila Rojas Valderrama; Jaime Sáez Quiroz; Consuelo Veloso Ávila</t>
         </is>
       </c>
     </row>
     <row r="10" ht="70" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>17.817-07</t>
+          <t>15.643-06</t>
         </is>
       </c>
       <c r="B10" s="11" t="inlineStr">
         <is>
-          <t>Moderniza el régimen normativo de las corporaciones y fundaciones, y fortalece su fiscalización</t>
+          <t>Modifica normas legales que indica para obligar a las organizaciones no gubernamentales a transparentar sus ingresos y mecanismos de financiamiento</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
@@ -1086,37 +1086,37 @@
       </c>
       <c r="D10" s="11" t="inlineStr">
         <is>
-          <t>Primer trámite constitucional / C.Diputados — Cuenta del Mensaje 122-374 que hace presente la urgencia Simple</t>
+          <t>Segundo trámite constitucional / Senado — Cuenta del Mensaje 123-374 que retira y hace presente la urgencia Simple</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>Simple</t>
+          <t>Sin urgencia</t>
         </is>
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>Cámara</t>
+          <t>Senado</t>
         </is>
       </c>
       <c r="G10" s="11" t="inlineStr">
         <is>
-          <t>Constitución, Legislación, Justicia y Reglamento</t>
+          <t>Gobierno, Descentralización y Regionalización</t>
         </is>
       </c>
       <c r="H10" s="4" t="inlineStr">
         <is>
-          <t>8 de septiembre de 2025</t>
+          <t>3 de enero de 2023</t>
         </is>
       </c>
       <c r="I10" s="11" t="inlineStr">
         <is>
-          <t>Primer trámite constitucional / C.Diputados</t>
+          <t>Segundo trámite constitucional / Senado</t>
         </is>
       </c>
       <c r="J10" s="4" t="inlineStr">
         <is>
-          <t>Mensaje</t>
+          <t>Moción</t>
         </is>
       </c>
       <c r="K10" s="4" t="inlineStr">
@@ -1126,29 +1126,29 @@
       </c>
       <c r="L10" s="11" t="inlineStr">
         <is>
-          <t>Ministerio de Justicia y Derechos Humanos</t>
+          <t>Miguel Ángel Calisto Águila; Erika Olivera De La Fuente; Joanna Pérez Olea; Jorge Saffirio Espinoza; Leonardo Soto Ferrada</t>
         </is>
       </c>
     </row>
     <row r="11" ht="70" customHeight="1">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>16.888-06</t>
+          <t>17.817-07</t>
         </is>
       </c>
       <c r="B11" s="12" t="inlineStr">
         <is>
-          <t>Moderniza la regulación del lobby y las gestiones de intereses particulares ante las autoridades y funcionarios</t>
+          <t>Moderniza el régimen normativo de las corporaciones y fundaciones, y fortalece su fiscalización</t>
         </is>
       </c>
       <c r="C11" s="7" t="inlineStr">
         <is>
-          <t>13/05/2026</t>
+          <t>02/06/2026</t>
         </is>
       </c>
       <c r="D11" s="12" t="inlineStr">
         <is>
-          <t>Primer trámite constitucional / C.Diputados — Discusión general . Queda pendiente</t>
+          <t>Primer trámite constitucional / C.Diputados — Cuenta del Mensaje 122-374 que hace presente la urgencia Simple</t>
         </is>
       </c>
       <c r="E11" s="7" t="inlineStr">
@@ -1163,17 +1163,17 @@
       </c>
       <c r="G11" s="12" t="inlineStr">
         <is>
-          <t>En Sala</t>
+          <t>Constitución, Legislación, Justicia y Reglamento</t>
         </is>
       </c>
       <c r="H11" s="7" t="inlineStr">
         <is>
-          <t>31 de mayo de 2024</t>
+          <t>8 de septiembre de 2025</t>
         </is>
       </c>
       <c r="I11" s="12" t="inlineStr">
         <is>
-          <t>Primer trámite constitucional / C.Diputados — Diario</t>
+          <t>Primer trámite constitucional / C.Diputados</t>
         </is>
       </c>
       <c r="J11" s="7" t="inlineStr">
@@ -1188,29 +1188,29 @@
       </c>
       <c r="L11" s="12" t="inlineStr">
         <is>
-          <t>Ministerio Secretaría General de Gobierno; Ministerio Secretaría General de la Presidencia; Ministerio de Hacienda; Ministerio de Justicia y Derechos Humanos</t>
+          <t>Ministerio de Justicia y Derechos Humanos</t>
         </is>
       </c>
     </row>
     <row r="12" ht="70" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>16746-06</t>
+          <t>16.888-06</t>
         </is>
       </c>
       <c r="B12" s="11" t="inlineStr">
         <is>
-          <t>Modifica la ley N° 20.285, sobre acceso a la informacion pública, para elevar los estándares de transparencia corporativa exigible a las empresas públicas</t>
+          <t>Moderniza la regulación del lobby y las gestiones de intereses particulares ante las autoridades y funcionarios</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>23/03/2026</t>
+          <t>13/05/2026</t>
         </is>
       </c>
       <c r="D12" s="11" t="inlineStr">
         <is>
-          <t>Primer trámite constitucional / C.Diputados — Cuenta del Mensaje 14-374 que hace presente la urgencia Simple</t>
+          <t>Primer trámite constitucional / C.Diputados — Discusión general . Queda pendiente</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr">
@@ -1225,59 +1225,59 @@
       </c>
       <c r="G12" s="11" t="inlineStr">
         <is>
-          <t>Gobierno Interior Nacionalidad Ciudadanía y Regionalización</t>
+          <t>En Sala</t>
         </is>
       </c>
       <c r="H12" s="4" t="inlineStr">
         <is>
-          <t>Miércoles 10 de Abril, 2024</t>
+          <t>31 de mayo de 2024</t>
         </is>
       </c>
       <c r="I12" s="11" t="inlineStr">
         <is>
-          <t>Primer trámite constitucional / C.Diputados</t>
+          <t>Primer trámite constitucional / C.Diputados — Diario</t>
         </is>
       </c>
       <c r="J12" s="4" t="inlineStr">
         <is>
-          <t>Moción</t>
+          <t>Mensaje</t>
         </is>
       </c>
       <c r="K12" s="4" t="inlineStr">
         <is>
-          <t>C.Diputados</t>
+          <t>Cámara de Diputados</t>
         </is>
       </c>
       <c r="L12" s="11" t="inlineStr">
         <is>
-          <t>Becker Alvear, Miguel Ángel; Berger Fett, Bernardo; Castro Bascuñán, José Miguel; Fuenzalida Cobo, Juan; Jouannet Valderrama, Andrés; Matheson Villán, Christian; Meza Pereira, José Carlos; Tapia Ramos, Cristián; Weisse Novoa, Flor</t>
+          <t>Ministerio Secretaría General de Gobierno; Ministerio Secretaría General de la Presidencia; Ministerio de Hacienda; Ministerio de Justicia y Derechos Humanos</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>17.797-06</t>
+          <t>16746-06</t>
         </is>
       </c>
       <c r="B13" s="12" t="inlineStr">
         <is>
-          <t>Modifica la ley N° 20.500, sobre Asociaciones y Participación Ciudadana en la Gestión Pública, y otros cuerpos normativos que indica</t>
+          <t>Modifica la ley N° 20.285, sobre acceso a la informacion pública, para elevar los estándares de transparencia corporativa exigible a las empresas públicas</t>
         </is>
       </c>
       <c r="C13" s="7" t="inlineStr">
         <is>
-          <t>02/03/2026</t>
+          <t>23/03/2026</t>
         </is>
       </c>
       <c r="D13" s="12" t="inlineStr">
         <is>
-          <t>Primer trámite constitucional / C.Diputados — Cuenta del Mensaje 1602-373 que hace presente la urgencia Suma</t>
+          <t>Primer trámite constitucional / C.Diputados — Cuenta del Mensaje 14-374 que hace presente la urgencia Simple</t>
         </is>
       </c>
       <c r="E13" s="7" t="inlineStr">
         <is>
-          <t>Suma</t>
+          <t>Simple</t>
         </is>
       </c>
       <c r="F13" s="7" t="inlineStr">
@@ -1292,7 +1292,7 @@
       </c>
       <c r="H13" s="7" t="inlineStr">
         <is>
-          <t>1 de septiembre de 2025</t>
+          <t>Miércoles 10 de Abril, 2024</t>
         </is>
       </c>
       <c r="I13" s="12" t="inlineStr">
@@ -1302,69 +1302,69 @@
       </c>
       <c r="J13" s="7" t="inlineStr">
         <is>
-          <t>Mensaje</t>
+          <t>Moción</t>
         </is>
       </c>
       <c r="K13" s="7" t="inlineStr">
         <is>
-          <t>Cámara de Diputados</t>
+          <t>C.Diputados</t>
         </is>
       </c>
       <c r="L13" s="12" t="inlineStr">
         <is>
-          <t>Ministerio Secretaría General de Gobierno</t>
+          <t>Becker Alvear, Miguel Ángel; Berger Fett, Bernardo; Castro Bascuñán, José Miguel; Fuenzalida Cobo, Juan; Jouannet Valderrama, Andrés; Matheson Villán, Christian; Meza Pereira, José Carlos; Tapia Ramos, Cristián; Weisse Novoa, Flor</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>16.886-12</t>
+          <t>17.797-06</t>
         </is>
       </c>
       <c r="B14" s="11" t="inlineStr">
         <is>
-          <t>Dicta normas sobre protección de personas defensoras de la naturaleza y los derechos humanos medioambientales</t>
+          <t>Modifica la ley N° 20.500, sobre Asociaciones y Participación Ciudadana en la Gestión Pública, y otros cuerpos normativos que indica</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>08/10/2025</t>
+          <t>02/03/2026</t>
         </is>
       </c>
       <c r="D14" s="11" t="inlineStr">
         <is>
-          <t>Segundo trámite constitucional / Senado — Cuenta de proyecto . Pasa a Comisión de Derechos Humanos, Nacionalidad y Ciudadanía</t>
+          <t>Primer trámite constitucional / C.Diputados — Cuenta del Mensaje 1602-373 que hace presente la urgencia Suma</t>
         </is>
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>Sin urgencia</t>
+          <t>Suma</t>
         </is>
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>Senado</t>
+          <t>Cámara</t>
         </is>
       </c>
       <c r="G14" s="11" t="inlineStr">
         <is>
-          <t>Derechos Humanos, Nacionalidad y Ciudadanía</t>
+          <t>Gobierno Interior Nacionalidad Ciudadanía y Regionalización</t>
         </is>
       </c>
       <c r="H14" s="4" t="inlineStr">
         <is>
-          <t>29 de mayo de 2024</t>
+          <t>1 de septiembre de 2025</t>
         </is>
       </c>
       <c r="I14" s="11" t="inlineStr">
         <is>
-          <t>Segundo trámite constitucional / Senado</t>
+          <t>Primer trámite constitucional / C.Diputados</t>
         </is>
       </c>
       <c r="J14" s="4" t="inlineStr">
         <is>
-          <t>Moción</t>
+          <t>Mensaje</t>
         </is>
       </c>
       <c r="K14" s="4" t="inlineStr">
@@ -1374,29 +1374,29 @@
       </c>
       <c r="L14" s="11" t="inlineStr">
         <is>
-          <t>Alejandro Bernales; Viviana Delgado; Luis Malla (A); Vlado Mirosevic; Sebastián Videla</t>
+          <t>Ministerio Secretaría General de Gobierno</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>17.520-17</t>
+          <t>16.886-12</t>
         </is>
       </c>
       <c r="B15" s="12" t="inlineStr">
         <is>
-          <t>Establece la obligación de incorporar la debida diligencia en derechos humanos a las empresas que operen en territorio nacional</t>
+          <t>Dicta normas sobre protección de personas defensoras de la naturaleza y los derechos humanos medioambientales</t>
         </is>
       </c>
       <c r="C15" s="7" t="inlineStr">
         <is>
-          <t>07/05/2025</t>
+          <t>08/10/2025</t>
         </is>
       </c>
       <c r="D15" s="12" t="inlineStr">
         <is>
-          <t>Primer trámite constitucional / C.Diputados — Oficio N° 20406. Deriva a la Comisión de Economía, Fomento; Micro, Pequeña y Mediana Empresa; Protección de los Consumidores y Turismo, el proyecto de ley asignado inicialmente a la Comisión de Derechos Humanos.</t>
+          <t>Segundo trámite constitucional / Senado — Cuenta de proyecto . Pasa a Comisión de Derechos Humanos, Nacionalidad y Ciudadanía</t>
         </is>
       </c>
       <c r="E15" s="7" t="inlineStr">
@@ -1406,22 +1406,22 @@
       </c>
       <c r="F15" s="7" t="inlineStr">
         <is>
-          <t>Cámara</t>
+          <t>Senado</t>
         </is>
       </c>
       <c r="G15" s="12" t="inlineStr">
         <is>
-          <t>Derechos Humanos y Pueblos Originarios</t>
+          <t>Derechos Humanos, Nacionalidad y Ciudadanía</t>
         </is>
       </c>
       <c r="H15" s="7" t="inlineStr">
         <is>
-          <t>5 de mayo de 2025</t>
+          <t>29 de mayo de 2024</t>
         </is>
       </c>
       <c r="I15" s="12" t="inlineStr">
         <is>
-          <t>Primer trámite constitucional / C.Diputados — Oficio</t>
+          <t>Segundo trámite constitucional / Senado</t>
         </is>
       </c>
       <c r="J15" s="7" t="inlineStr">
@@ -1436,29 +1436,29 @@
       </c>
       <c r="L15" s="12" t="inlineStr">
         <is>
-          <t>María Francisca Bello Campos; Roberto Celedón Fernández; Lorena Fries Monleón; Andrés Giordano Salazar; Diego Ibáñez Cotroneo; Camila Rojas Valderrama; Jaime Sáez Quiroz; Clara Sagardia Cabezas; Carolina Tello Rojas; Gael Yeomans Araya</t>
+          <t>Alejandro Bernales; Viviana Delgado; Luis Malla (A); Vlado Mirosevic; Sebastián Videla</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>17.446-17</t>
+          <t>17.520-17</t>
         </is>
       </c>
       <c r="B16" s="11" t="inlineStr">
         <is>
-          <t>Establece y regula la debida diligencia de las empresas en el respeto a los derechos humanos, el medio ambiente y el cambio climático</t>
+          <t>Establece la obligación de incorporar la debida diligencia en derechos humanos a las empresas que operen en territorio nacional</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>08/04/2025</t>
+          <t>07/05/2025</t>
         </is>
       </c>
       <c r="D16" s="11" t="inlineStr">
         <is>
-          <t>Primer trámite constitucional / Senado — Cuenta de proyecto . Pasa a Comisión de Derechos Humanos, Nacionalidad y Ciudadanía</t>
+          <t>Primer trámite constitucional / C.Diputados — Oficio N° 20406. Deriva a la Comisión de Economía, Fomento; Micro, Pequeña y Mediana Empresa; Protección de los Consumidores y Turismo, el proyecto de ley asignado inicialmente a la Comisión de Derechos Humanos.</t>
         </is>
       </c>
       <c r="E16" s="4" t="inlineStr">
@@ -1468,22 +1468,22 @@
       </c>
       <c r="F16" s="4" t="inlineStr">
         <is>
-          <t>Senado</t>
+          <t>Cámara</t>
         </is>
       </c>
       <c r="G16" s="11" t="inlineStr">
         <is>
-          <t>Derechos Humanos, Nacionalidad y Ciudadanía</t>
+          <t>Derechos Humanos y Pueblos Originarios</t>
         </is>
       </c>
       <c r="H16" s="4" t="inlineStr">
         <is>
-          <t>3 de abril de 2025</t>
+          <t>5 de mayo de 2025</t>
         </is>
       </c>
       <c r="I16" s="11" t="inlineStr">
         <is>
-          <t>Primer trámite constitucional / Senado</t>
+          <t>Primer trámite constitucional / C.Diputados — Oficio</t>
         </is>
       </c>
       <c r="J16" s="4" t="inlineStr">
@@ -1493,72 +1493,134 @@
       </c>
       <c r="K16" s="4" t="inlineStr">
         <is>
-          <t>Senado</t>
+          <t>Cámara de Diputados</t>
         </is>
       </c>
       <c r="L16" s="11" t="inlineStr">
         <is>
-          <t>Isabel Allende Bussi</t>
+          <t>María Francisca Bello Campos; Roberto Celedón Fernández; Lorena Fries Monleón; Andrés Giordano Salazar; Diego Ibáñez Cotroneo; Camila Rojas Valderrama; Jaime Sáez Quiroz; Clara Sagardia Cabezas; Carolina Tello Rojas; Gael Yeomans Araya</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
         <is>
+          <t>17.446-17</t>
+        </is>
+      </c>
+      <c r="B17" s="12" t="inlineStr">
+        <is>
+          <t>Establece y regula la debida diligencia de las empresas en el respeto a los derechos humanos, el medio ambiente y el cambio climático</t>
+        </is>
+      </c>
+      <c r="C17" s="7" t="inlineStr">
+        <is>
+          <t>08/04/2025</t>
+        </is>
+      </c>
+      <c r="D17" s="12" t="inlineStr">
+        <is>
+          <t>Primer trámite constitucional / Senado — Cuenta de proyecto . Pasa a Comisión de Derechos Humanos, Nacionalidad y Ciudadanía</t>
+        </is>
+      </c>
+      <c r="E17" s="7" t="inlineStr">
+        <is>
+          <t>Sin urgencia</t>
+        </is>
+      </c>
+      <c r="F17" s="7" t="inlineStr">
+        <is>
+          <t>Senado</t>
+        </is>
+      </c>
+      <c r="G17" s="12" t="inlineStr">
+        <is>
+          <t>Derechos Humanos, Nacionalidad y Ciudadanía</t>
+        </is>
+      </c>
+      <c r="H17" s="7" t="inlineStr">
+        <is>
+          <t>3 de abril de 2025</t>
+        </is>
+      </c>
+      <c r="I17" s="12" t="inlineStr">
+        <is>
+          <t>Primer trámite constitucional / Senado</t>
+        </is>
+      </c>
+      <c r="J17" s="7" t="inlineStr">
+        <is>
+          <t>Moción</t>
+        </is>
+      </c>
+      <c r="K17" s="7" t="inlineStr">
+        <is>
+          <t>Senado</t>
+        </is>
+      </c>
+      <c r="L17" s="12" t="inlineStr">
+        <is>
+          <t>Isabel Allende Bussi</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
           <t>17196-17</t>
         </is>
       </c>
-      <c r="B17" s="12" t="inlineStr">
+      <c r="B18" s="11" t="inlineStr">
         <is>
           <t>Modifica la ley N° 18.046, Ley sobre Sociedades Anónimas, con el objeto de establecer obligaciones para promover la protección de derechos humanos, a las personas jurídicas que indica.</t>
         </is>
       </c>
-      <c r="C17" s="7" t="inlineStr">
+      <c r="C18" s="4" t="inlineStr">
         <is>
           <t>21/10/2024</t>
         </is>
       </c>
-      <c r="D17" s="12" t="inlineStr">
+      <c r="D18" s="11" t="inlineStr">
         <is>
           <t>Primer trámite constitucional / Senado — Cuenta de proyecto . Pasa a Comisión de Derechos Humanos, Nacionalidad y Ciudadanía</t>
         </is>
       </c>
-      <c r="E17" s="7" t="inlineStr">
+      <c r="E18" s="4" t="inlineStr">
         <is>
           <t>Sin urgencia</t>
         </is>
       </c>
-      <c r="F17" s="7" t="inlineStr">
+      <c r="F18" s="4" t="inlineStr">
         <is>
           <t>Senado</t>
         </is>
       </c>
-      <c r="G17" s="12" t="inlineStr">
+      <c r="G18" s="11" t="inlineStr">
         <is>
           <t>Derechos Humanos, Nacionalidad y Ciudadanía</t>
         </is>
       </c>
-      <c r="H17" s="7" t="inlineStr">
+      <c r="H18" s="4" t="inlineStr">
         <is>
           <t>Lunes 21 de Octubre, 2024</t>
         </is>
       </c>
-      <c r="I17" s="12" t="inlineStr">
+      <c r="I18" s="11" t="inlineStr">
         <is>
           <t>Primer trámite constitucional / Senado</t>
         </is>
       </c>
-      <c r="J17" s="7" t="inlineStr">
+      <c r="J18" s="4" t="inlineStr">
         <is>
           <t>Moción</t>
         </is>
       </c>
-      <c r="K17" s="7" t="inlineStr">
+      <c r="K18" s="4" t="inlineStr">
         <is>
           <t>Senado</t>
         </is>
       </c>
-      <c r="L17" s="12" t="inlineStr">
+      <c r="L18" s="11" t="inlineStr">
         <is>
           <t>Vodanovic Rojas, Paulina</t>
         </is>
@@ -1582,6 +1644,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A15" r:id="rId14"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A16" r:id="rId15"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A17" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A18" r:id="rId17"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: actualización semanal 2026-10-26
</commit_message>
<xml_diff>
--- a/seguimiento_legislativo.xlsx
+++ b/seguimiento_legislativo.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Seguimiento Legislativo" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Seguimiento Legislativo" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -729,7 +729,7 @@
       </c>
       <c r="G4" s="11" t="inlineStr">
         <is>
-          <t>En espera de promulgación</t>
+          <t>Ley N° 21.850 (Diario Oficial del 17/10/2026)</t>
         </is>
       </c>
       <c r="H4" s="4" t="inlineStr">

</xml_diff>